<commit_message>
edito archivo .xlsx x2
</commit_message>
<xml_diff>
--- a/documentos/EMBALAJES ETIQUETAS KIWI.xlsx
+++ b/documentos/EMBALAJES ETIQUETAS KIWI.xlsx
@@ -1,31 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30502"/>
-  <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{45379966-0D0C-46F8-93F0-2EA660075C21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+  <fileVersion appName="Calc" lowestEdited="7"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191028" iterateDelta="1E-4"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -36,599 +22,603 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="882" uniqueCount="196">
   <si>
-    <t>ESPECIE</t>
-  </si>
-  <si>
-    <t>COLOR</t>
-  </si>
-  <si>
-    <t>EMBALAJE</t>
-  </si>
-  <si>
-    <t>CATEGORÍA</t>
-  </si>
-  <si>
-    <t>PLU</t>
-  </si>
-  <si>
-    <t>DESTINO</t>
-  </si>
-  <si>
-    <t>CLIENTE</t>
-  </si>
-  <si>
-    <t>ENVASE</t>
-  </si>
-  <si>
-    <t>BOLSA</t>
-  </si>
-  <si>
-    <t>OPCIONAL 2</t>
-  </si>
-  <si>
-    <t>EXTRA</t>
-  </si>
-  <si>
-    <t>SORELI</t>
-  </si>
-  <si>
-    <t>EF</t>
-  </si>
-  <si>
-    <t>10S</t>
-  </si>
-  <si>
-    <t>AMARILLO 3279</t>
-  </si>
-  <si>
-    <t>ROTTERDAM/LATAM</t>
-  </si>
-  <si>
-    <t>HILL/TBC</t>
-  </si>
-  <si>
-    <t>NORMAL</t>
-  </si>
-  <si>
-    <t>SPECIAL CARGO 938</t>
-  </si>
-  <si>
-    <t>D9S</t>
-  </si>
-  <si>
-    <t>NO</t>
-  </si>
-  <si>
-    <t>TODOS</t>
-  </si>
-  <si>
-    <t>PERFORADA 0.9%</t>
-  </si>
-  <si>
-    <t>10C</t>
-  </si>
-  <si>
-    <t>MÉXICO</t>
-  </si>
-  <si>
-    <t>FRFI</t>
-  </si>
-  <si>
-    <t>T6C</t>
-  </si>
-  <si>
-    <t>INGLATERRA</t>
-  </si>
-  <si>
-    <t>DPSL (TESCO)</t>
-  </si>
-  <si>
-    <t>CAJA TESCO</t>
-  </si>
-  <si>
-    <t>1BS</t>
-  </si>
-  <si>
-    <t>ESPAÑA</t>
-  </si>
-  <si>
-    <t>EUBA</t>
-  </si>
-  <si>
-    <t>BANDEJA</t>
-  </si>
-  <si>
-    <t>9CS</t>
-  </si>
-  <si>
-    <t>U.S.A.</t>
-  </si>
-  <si>
-    <t>TRUCCO</t>
-  </si>
-  <si>
-    <t>NORMAL/CAJA PARA UVA</t>
-  </si>
-  <si>
-    <t>CLAMSHELL</t>
-  </si>
-  <si>
-    <t>EA</t>
-  </si>
-  <si>
-    <t>LATINOAMÉRICA</t>
-  </si>
-  <si>
-    <t>SUNXY (HFY02)</t>
-  </si>
-  <si>
-    <t>ESPAÑA/ITALIA/EUROPA</t>
-  </si>
-  <si>
-    <t>EUBA/DOIT/TBN</t>
-  </si>
-  <si>
-    <t>DOLE</t>
-  </si>
-  <si>
-    <t>SPECIAL CARGO 839</t>
-  </si>
-  <si>
-    <t>1BG</t>
-  </si>
-  <si>
-    <t>ESPAÑA /ITALIA/EUROPA</t>
-  </si>
-  <si>
-    <t>LOPE/TITA/TBN</t>
-  </si>
-  <si>
-    <t>TBN</t>
-  </si>
-  <si>
-    <t>PERFORADA 0,9%</t>
-  </si>
-  <si>
-    <t>10c</t>
-  </si>
-  <si>
-    <t>HAYWARD</t>
-  </si>
-  <si>
-    <t>T1P</t>
-  </si>
-  <si>
-    <t>HOLANDA</t>
-  </si>
-  <si>
-    <t>NATG</t>
-  </si>
-  <si>
-    <t>CAJA PLÁSTICA</t>
-  </si>
-  <si>
-    <t>NATP</t>
-  </si>
-  <si>
-    <t>GRAMAJE ACOTADO</t>
-  </si>
-  <si>
-    <t>TPA</t>
-  </si>
-  <si>
-    <t>MAP</t>
-  </si>
-  <si>
-    <t>1SD</t>
-  </si>
-  <si>
-    <t>ASDA</t>
-  </si>
-  <si>
-    <t>T1C</t>
-  </si>
-  <si>
-    <t>DOLE 4030</t>
-  </si>
-  <si>
-    <t>BRASIL</t>
-  </si>
-  <si>
-    <t>TBC</t>
-  </si>
-  <si>
-    <t>06C</t>
-  </si>
-  <si>
-    <t>RUSIA</t>
-  </si>
-  <si>
-    <t>RVIN</t>
-  </si>
-  <si>
-    <t>D09</t>
-  </si>
-  <si>
-    <t>1CT</t>
-  </si>
-  <si>
-    <t>1SC</t>
-  </si>
-  <si>
-    <t>INGLATERRA/ITALIA/INGLATERRA/IRLANDA/HOLANDA/CANADA/INGLATERRA/INGLATERRA</t>
-  </si>
-  <si>
-    <t>GPAC/DOIT/TOTA/TOTI/NATG/TAST/TOTM/ROBS</t>
-  </si>
-  <si>
-    <t>ASM</t>
-  </si>
-  <si>
-    <t>/</t>
-  </si>
-  <si>
-    <t>TOTM</t>
-  </si>
-  <si>
-    <t>1CP</t>
-  </si>
-  <si>
-    <t>PREWORLD</t>
-  </si>
-  <si>
-    <t>A1E</t>
-  </si>
-  <si>
-    <t>SIN CATEGORÍA ETIQUETA</t>
-  </si>
-  <si>
-    <t>ARE</t>
-  </si>
-  <si>
-    <t>4030 GENÉRICO</t>
-  </si>
-  <si>
-    <t>BARG</t>
-  </si>
-  <si>
-    <t>PRIMORE</t>
-  </si>
-  <si>
-    <t>A1P</t>
-  </si>
-  <si>
-    <t>INDIA/INDIA</t>
-  </si>
-  <si>
-    <t>FFAP/GTFR</t>
-  </si>
-  <si>
-    <t>A1C</t>
-  </si>
-  <si>
-    <t>ARGENTINA/PERÚ/INDIA</t>
-  </si>
-  <si>
-    <t>DNAT/PAEX-MANP/GTFR</t>
-  </si>
-  <si>
-    <t>ASC</t>
-  </si>
-  <si>
-    <t>INGLATERRA/INGLATERRA/INDIA/DINAMARCA/IRLANDA/IRLANDA/HOLANDA</t>
-  </si>
-  <si>
-    <t>GPAC/ROBINSON/FFAP/TOTN/TOTI NO TESCO/TOTI/EDEKA</t>
-  </si>
-  <si>
-    <t>A1H</t>
-  </si>
-  <si>
-    <t>SHARBATLY</t>
-  </si>
-  <si>
-    <t>ARABIA</t>
-  </si>
-  <si>
-    <t>ARP</t>
-  </si>
-  <si>
-    <t>INDIA</t>
-  </si>
-  <si>
-    <t>FTSY</t>
-  </si>
-  <si>
-    <t>ARS</t>
-  </si>
-  <si>
-    <t>R09</t>
-  </si>
-  <si>
-    <t>OPPY</t>
-  </si>
-  <si>
-    <t>1SR</t>
-  </si>
-  <si>
-    <t>LOPE</t>
-  </si>
-  <si>
-    <t>ASD</t>
-  </si>
-  <si>
-    <t>1BM</t>
-  </si>
-  <si>
-    <t>DINAMARCA</t>
-  </si>
-  <si>
-    <t>TOTN</t>
-  </si>
-  <si>
-    <t>1BC</t>
-  </si>
-  <si>
-    <t>1BH</t>
-  </si>
-  <si>
-    <t>3GD</t>
-  </si>
-  <si>
-    <t>3AM</t>
-  </si>
-  <si>
-    <t>2CB</t>
-  </si>
-  <si>
-    <t>WALMART</t>
-  </si>
-  <si>
-    <t>CAJA CAFÉ</t>
-  </si>
-  <si>
-    <t>SIN FECHA EN CLAMSHELL</t>
-  </si>
-  <si>
-    <t>9CB</t>
-  </si>
-  <si>
-    <t>9CW</t>
-  </si>
-  <si>
-    <t>2CT</t>
-  </si>
-  <si>
-    <t>CAJA VERDE</t>
-  </si>
-  <si>
-    <t>FECHA PACK DATE + 14 DÍAS (O SIN FECHA)</t>
-  </si>
-  <si>
-    <t>9CT</t>
-  </si>
-  <si>
-    <t>CAJA VERDE - CAFÉ</t>
-  </si>
-  <si>
-    <t>S12</t>
-  </si>
-  <si>
-    <t>SUNP</t>
-  </si>
-  <si>
-    <t>MIGHTIES</t>
-  </si>
-  <si>
-    <t>C12</t>
-  </si>
-  <si>
-    <t>1MT</t>
-  </si>
-  <si>
-    <t>MÉXICO/MÉXICO/MÉXICO/MÉXICO/MÉXICO/BRASIL/BRASIL/BRASIL</t>
-  </si>
-  <si>
-    <t>WAME/FRCL/ACUM/FRFI/AUST/CRIS/PERB/FSUL</t>
-  </si>
-  <si>
-    <t>MICROPERFORADA 0.3%</t>
-  </si>
-  <si>
-    <t>9CR</t>
-  </si>
-  <si>
-    <t>2CR</t>
-  </si>
-  <si>
-    <t>2PW</t>
-  </si>
-  <si>
-    <t>9PW</t>
-  </si>
-  <si>
-    <t>14P</t>
-  </si>
-  <si>
-    <t>CHILE</t>
-  </si>
-  <si>
-    <t>RENTAPACK</t>
-  </si>
-  <si>
-    <t>10T</t>
-  </si>
-  <si>
-    <t>ACUM/FRCL</t>
-  </si>
-  <si>
-    <t>PAPEL CAMISA</t>
-  </si>
-  <si>
-    <t>WAME</t>
-  </si>
-  <si>
-    <t>ACP</t>
-  </si>
-  <si>
-    <t>BRASIL/MÉXICO/BRASIL/BRASIL/BRASIL/MÉXICO/BRASIL/MÉXICO/MÉXICO</t>
-  </si>
-  <si>
-    <t>TBC/ACUM/LPDI/CRIS/PERB/FRFI/FSUL/AUST/WAME</t>
-  </si>
-  <si>
-    <t>APE</t>
-  </si>
-  <si>
-    <t>ETIQUETA PRIMORE</t>
-  </si>
-  <si>
-    <t>ASP</t>
-  </si>
-  <si>
-    <t>CALIBRE 46 Y SIN CAT2</t>
-  </si>
-  <si>
-    <t>A1R</t>
-  </si>
-  <si>
-    <t>N1L</t>
-  </si>
-  <si>
-    <t>CANADÁ</t>
-  </si>
-  <si>
-    <t>LOBL</t>
-  </si>
-  <si>
-    <t>NEGRA</t>
-  </si>
-  <si>
-    <t>FECHA JULIANA</t>
-  </si>
-  <si>
-    <t>1CL</t>
-  </si>
-  <si>
-    <t>VERDE</t>
-  </si>
-  <si>
-    <t>CHILE/URUGUAY</t>
-  </si>
-  <si>
-    <t>CENCOSUD/PROX</t>
-  </si>
-  <si>
-    <t>A9C</t>
-  </si>
-  <si>
-    <t>GOFP</t>
-  </si>
-  <si>
-    <t>T1A</t>
-  </si>
-  <si>
-    <t>PERÚ/COLOMBIA</t>
-  </si>
-  <si>
-    <t>ESAL/FDCO</t>
-  </si>
-  <si>
-    <t>INGLATERRA/INGLATERRA/R. DOMINICANA</t>
-  </si>
-  <si>
-    <t>GPAC/ROBINSON/MEJI</t>
-  </si>
-  <si>
-    <t>ARE (A1R)</t>
-  </si>
-  <si>
-    <t>9MW (9CV)</t>
-  </si>
-  <si>
-    <t>2MW (2CV)</t>
-  </si>
-  <si>
-    <t>C22</t>
-  </si>
-  <si>
-    <t>CLAMSHELL ETIQUETA DOLE</t>
-  </si>
-  <si>
-    <t>S22</t>
-  </si>
-  <si>
-    <t>CLANSHELL SIN ETIQUETA</t>
-  </si>
-  <si>
-    <t>1SB</t>
-  </si>
-  <si>
-    <t>ASC (1SC)</t>
-  </si>
-  <si>
-    <t>B12</t>
-  </si>
-  <si>
-    <t>1MT (1CT)</t>
-  </si>
-  <si>
-    <t>CE</t>
-  </si>
-  <si>
-    <t>14K</t>
-  </si>
-  <si>
-    <t>MERCADO INTERNO</t>
-  </si>
-  <si>
-    <t>B10</t>
-  </si>
-  <si>
-    <t>TOTTUS</t>
-  </si>
-  <si>
-    <t>RENTAPACK BOLSITAS</t>
-  </si>
-  <si>
-    <t>10 BOLSAS 1 KG</t>
-  </si>
-  <si>
-    <t>10P</t>
-  </si>
-  <si>
-    <t>LITUANIA</t>
-  </si>
-  <si>
-    <t>VTA/INTER</t>
-  </si>
-  <si>
-    <t>6 BOLSAS 2 KG</t>
-  </si>
-  <si>
-    <t>BW1</t>
-  </si>
-  <si>
-    <t>SUPERMERCADO</t>
-  </si>
-  <si>
-    <t>12 BOLSAS 1 KG</t>
-  </si>
-  <si>
-    <t>BS1</t>
-  </si>
-  <si>
-    <t>RIÑÓN</t>
-  </si>
-  <si>
-    <t>10X</t>
+    <t xml:space="preserve">ESPECIE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMBALAJE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CATEGORÍA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DESTINO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLIENTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENVASE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BOLSA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PESO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXTRA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SORELI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMARILLO 3279</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROTTERDAM/LATAM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HILL/TBC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NORMAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SPECIAL CARGO 938</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D9S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TODOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PERFORADA 0.9%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MÉXICO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FRFI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T6C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INGLATERRA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DPSL (TESCO)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAJA TESCO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1BS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESPAÑA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUBA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BANDEJA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9CS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U.S.A.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRUCCO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NORMAL/CAJA PARA UVA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLAMSHELL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LATINOAMÉRICA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUNXY (HFY02)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESPAÑA/ITALIA/EUROPA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUBA/DOIT/TBN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SPECIAL CARGO 839</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1BG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESPAÑA /ITALIA/EUROPA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOPE/TITA/TBN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TBN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PERFORADA 0,9%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HAYWARD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T1P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HOLANDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NATG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAJA PLÁSTICA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NATP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GRAMAJE ACOTADO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TPA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1SD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T1C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOLE 4030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BRASIL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TBC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RUSIA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RVIN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1CT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1SC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INGLATERRA/ITALIA/INGLATERRA/IRLANDA/HOLANDA/CANADA/INGLATERRA/INGLATERRA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPAC/DOIT/TOTA/TOTI/NATG/TAST/TOTM/ROBS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1CP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PREWORLD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A1E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SIN CATEGORÍA ETIQUETA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4030 GENÉRICO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BARG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRIMORE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A1P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INDIA/INDIA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FFAP/GTFR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A1C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARGENTINA/PERÚ/INDIA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DNAT/PAEX-MANP/GTFR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INGLATERRA/INGLATERRA/INDIA/DINAMARCA/IRLANDA/IRLANDA/HOLANDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPAC/ROBINSON/FFAP/TOTN/TOTI NO TESCO/TOTI/EDEKA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A1H</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SHARBATLY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARABIA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INDIA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FTSY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPPY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1SR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOPE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1BM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DINAMARCA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1BC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1BH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3GD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3AM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2CB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WALMART</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAJA CAFÉ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SIN FECHA EN CLAMSHELL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9CB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9CW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2CT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAJA VERDE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FECHA PACK DATE + 14 DÍAS (O SIN FECHA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9CT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAJA VERDE - CAFÉ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUNP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MIGHTIES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1MT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MÉXICO/MÉXICO/MÉXICO/MÉXICO/MÉXICO/BRASIL/BRASIL/BRASIL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WAME/FRCL/ACUM/FRFI/AUST/CRIS/PERB/FSUL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MICROPERFORADA 0.3%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9CR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2CR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2PW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9PW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHILE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RENTAPACK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACUM/FRCL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PAPEL CAMISA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BRASIL/MÉXICO/BRASIL/BRASIL/BRASIL/MÉXICO/BRASIL/MÉXICO/MÉXICO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TBC/ACUM/LPDI/CRIS/PERB/FRFI/FSUL/AUST/WAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">APE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ETIQUETA PRIMORE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CALIBRE 46 Y SIN CAT2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A1R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N1L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CANADÁ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOBL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEGRA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FECHA JULIANA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1CL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VERDE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHILE/URUGUAY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CENCOSUD/PROX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A9C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOFP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T1A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PERÚ/COLOMBIA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESAL/FDCO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INGLATERRA/INGLATERRA/R. DOMINICANA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPAC/ROBINSON/MEJI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARE (A1R)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9MW (9CV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2MW (2CV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLAMSHELL ETIQUETA DOLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLANSHELL SIN ETIQUETA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1SB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASC (1SC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1MT (1CT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MERCADO INTERNO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTTUS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RENTAPACK BOLSITAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 BOLSAS 1 KG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LITUANIA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VTA/INTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 BOLSAS 2 KG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BW1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUPERMERCADO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 BOLSAS 1 KG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BS1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RIÑÓN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10X</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="#,##0"/>
+  </numFmts>
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -637,7 +627,22 @@
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -654,110 +659,123 @@
     </fill>
   </fills>
   <borders count="4">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
       <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="20">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
   <cellXfs count="12">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office 2013 - Tema de 2022">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -799,12 +817,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -836,7 +854,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -860,7 +878,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -920,79 +938,80 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A2:K121"/>
-  <sheetFormatPr defaultColWidth="10.5703125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="10.57421875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="16.28515625" customWidth="1"/>
-    <col min="2" max="2" width="6.85546875" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" customWidth="1"/>
-    <col min="5" max="5" width="14.85546875" customWidth="1"/>
-    <col min="6" max="6" width="87.5703125" customWidth="1"/>
-    <col min="7" max="7" width="54.5703125" customWidth="1"/>
-    <col min="8" max="8" width="23.140625" customWidth="1"/>
-    <col min="9" max="9" width="23" customWidth="1"/>
-    <col min="10" max="10" width="12.42578125" customWidth="1"/>
-    <col min="11" max="11" width="39.28515625" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="6.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="87.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="54.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="23.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="12.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="39.28"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:11">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="3" spans="1:11">
-      <c r="A3" s="1" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="1" t="s">
+      <c r="B3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="I3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="K3" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>11</v>
       </c>
@@ -1002,7 +1021,7 @@
       <c r="C4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E4" s="3" t="s">
@@ -1020,12 +1039,12 @@
       <c r="I4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="4">
+      <c r="J4" s="4" t="n">
         <v>10700</v>
       </c>
       <c r="K4" s="3"/>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
         <v>11</v>
       </c>
@@ -1035,7 +1054,7 @@
       <c r="C5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E5" s="3" t="s">
@@ -1056,7 +1075,7 @@
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
         <v>11</v>
       </c>
@@ -1066,7 +1085,7 @@
       <c r="C6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="3" t="s">
@@ -1087,7 +1106,7 @@
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
         <v>11</v>
       </c>
@@ -1097,7 +1116,7 @@
       <c r="C7" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="3" t="s">
@@ -1115,12 +1134,12 @@
       <c r="I7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J7" s="4">
+      <c r="J7" s="4" t="n">
         <v>6600</v>
       </c>
       <c r="K7" s="3"/>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
         <v>11</v>
       </c>
@@ -1130,7 +1149,7 @@
       <c r="C8" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E8" s="3" t="s">
@@ -1148,14 +1167,14 @@
       <c r="I8" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J8" s="4">
+      <c r="J8" s="4" t="n">
         <v>3500</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
@@ -1165,7 +1184,7 @@
       <c r="C9" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E9" s="3" t="s">
@@ -1188,7 +1207,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -1201,7 +1220,7 @@
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
         <v>11</v>
       </c>
@@ -1211,7 +1230,7 @@
       <c r="C11" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E11" s="3" t="s">
@@ -1232,81 +1251,81 @@
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
     </row>
-    <row r="12" spans="1:11">
-      <c r="A12" s="1"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
-    </row>
-    <row r="13" spans="1:11">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-    </row>
-    <row r="14" spans="1:11">
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-    </row>
-    <row r="18" spans="1:11">
-      <c r="A18" s="1" t="s">
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C18" s="1" t="s">
+      <c r="B18" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D18" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="E18" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="F18" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="G18" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H18" s="1" t="s">
+      <c r="H18" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I18" s="1" t="s">
+      <c r="I18" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J18" s="1" t="s">
+      <c r="J18" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K18" s="1" t="s">
+      <c r="K18" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="15" customHeight="1">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
         <v>41</v>
       </c>
@@ -1316,7 +1335,7 @@
       <c r="C19" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D19" s="3">
+      <c r="D19" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E19" s="3" t="s">
@@ -1334,14 +1353,14 @@
       <c r="I19" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="J19" s="4">
+      <c r="J19" s="4" t="n">
         <v>3510</v>
       </c>
       <c r="K19" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="1:11">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
         <v>41</v>
       </c>
@@ -1351,7 +1370,7 @@
       <c r="C20" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="D20" s="3">
+      <c r="D20" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E20" s="3" t="s">
@@ -1369,14 +1388,14 @@
       <c r="I20" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="J20" s="4">
+      <c r="J20" s="4" t="n">
         <v>3480</v>
       </c>
       <c r="K20" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:11">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
         <v>41</v>
       </c>
@@ -1386,7 +1405,7 @@
       <c r="C21" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D21" s="3">
+      <c r="D21" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E21" s="3" t="s">
@@ -1404,12 +1423,12 @@
       <c r="I21" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="J21" s="4">
+      <c r="J21" s="4" t="n">
         <v>10690</v>
       </c>
       <c r="K21" s="3"/>
     </row>
-    <row r="22" spans="1:11">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
         <v>41</v>
       </c>
@@ -1419,7 +1438,7 @@
       <c r="C22" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="D22" s="3">
+      <c r="D22" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E22" s="3" t="s">
@@ -1437,50 +1456,50 @@
       <c r="I22" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="J22" s="4">
+      <c r="J22" s="4" t="n">
         <v>10690</v>
       </c>
       <c r="K22" s="3"/>
     </row>
-    <row r="25" spans="1:11">
-      <c r="I25" s="2"/>
-    </row>
-    <row r="26" spans="1:11">
-      <c r="A26" s="1" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I25" s="1"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C26" s="1" t="s">
+      <c r="B26" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D26" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="E26" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F26" s="1" t="s">
+      <c r="F26" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G26" s="1" t="s">
+      <c r="G26" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H26" s="1" t="s">
+      <c r="H26" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I26" s="1" t="s">
+      <c r="I26" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J26" s="1" t="s">
+      <c r="J26" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K26" s="1" t="s">
+      <c r="K26" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:11">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
         <v>52</v>
       </c>
@@ -1490,7 +1509,7 @@
       <c r="C27" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="D27" s="3">
+      <c r="D27" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E27" s="3" t="s">
@@ -1508,12 +1527,12 @@
       <c r="I27" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J27" s="4">
+      <c r="J27" s="4" t="n">
         <v>10470</v>
       </c>
       <c r="K27" s="3"/>
     </row>
-    <row r="28" spans="1:11">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
         <v>52</v>
       </c>
@@ -1523,7 +1542,7 @@
       <c r="C28" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="D28" s="3">
+      <c r="D28" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E28" s="3" t="s">
@@ -1541,14 +1560,14 @@
       <c r="I28" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J28" s="4">
+      <c r="J28" s="4" t="n">
         <v>10470</v>
       </c>
       <c r="K28" s="3" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="29" spans="1:11">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
         <v>52</v>
       </c>
@@ -1558,7 +1577,7 @@
       <c r="C29" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D29" s="3">
+      <c r="D29" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E29" s="3" t="s">
@@ -1576,12 +1595,12 @@
       <c r="I29" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J29" s="4">
+      <c r="J29" s="4" t="n">
         <v>10510</v>
       </c>
       <c r="K29" s="3"/>
     </row>
-    <row r="30" spans="1:11">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
         <v>52</v>
       </c>
@@ -1591,7 +1610,7 @@
       <c r="C30" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D30" s="3">
+      <c r="D30" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E30" s="3" t="s">
@@ -1609,12 +1628,12 @@
       <c r="I30" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J30" s="4">
+      <c r="J30" s="4" t="n">
         <v>10670</v>
       </c>
       <c r="K30" s="3"/>
     </row>
-    <row r="31" spans="1:11">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
         <v>52</v>
       </c>
@@ -1624,7 +1643,7 @@
       <c r="C31" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="D31" s="3">
+      <c r="D31" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E31" s="3" t="s">
@@ -1642,14 +1661,14 @@
       <c r="I31" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J31" s="4">
+      <c r="J31" s="4" t="n">
         <v>10755</v>
       </c>
       <c r="K31" s="3" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="32" spans="1:11">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
         <v>52</v>
       </c>
@@ -1659,7 +1678,7 @@
       <c r="C32" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D32" s="3">
+      <c r="D32" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E32" s="3" t="s">
@@ -1677,12 +1696,12 @@
       <c r="I32" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J32" s="4">
+      <c r="J32" s="4" t="n">
         <v>10755</v>
       </c>
       <c r="K32" s="3"/>
     </row>
-    <row r="33" spans="1:11">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
         <v>52</v>
       </c>
@@ -1692,7 +1711,7 @@
       <c r="C33" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D33" s="3">
+      <c r="D33" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E33" s="3" t="s">
@@ -1710,12 +1729,12 @@
       <c r="I33" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J33" s="4">
+      <c r="J33" s="4" t="n">
         <v>6540</v>
       </c>
       <c r="K33" s="3"/>
     </row>
-    <row r="34" spans="1:11">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
         <v>52</v>
       </c>
@@ -1725,7 +1744,7 @@
       <c r="C34" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="D34" s="3">
+      <c r="D34" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E34" s="3" t="s">
@@ -1743,12 +1762,12 @@
       <c r="I34" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J34" s="4">
+      <c r="J34" s="4" t="n">
         <v>10350</v>
       </c>
       <c r="K34" s="3"/>
     </row>
-    <row r="35" spans="1:11">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
         <v>52</v>
       </c>
@@ -1758,7 +1777,7 @@
       <c r="C35" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D35" s="3">
+      <c r="D35" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E35" s="3" t="s">
@@ -1776,12 +1795,12 @@
       <c r="I35" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J35" s="4">
+      <c r="J35" s="4" t="n">
         <v>10755</v>
       </c>
       <c r="K35" s="3"/>
     </row>
-    <row r="36" spans="1:11">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
         <v>52</v>
       </c>
@@ -1791,7 +1810,7 @@
       <c r="C36" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="D36" s="3">
+      <c r="D36" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E36" s="3" t="s">
@@ -1809,12 +1828,12 @@
       <c r="I36" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J36" s="4">
+      <c r="J36" s="4" t="n">
         <v>10755</v>
       </c>
       <c r="K36" s="3"/>
     </row>
-    <row r="37" spans="1:11">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
         <v>52</v>
       </c>
@@ -1824,7 +1843,7 @@
       <c r="C37" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D37" s="3">
+      <c r="D37" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E37" s="3" t="s">
@@ -1842,12 +1861,12 @@
       <c r="I37" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J37" s="4">
+      <c r="J37" s="4" t="n">
         <v>10670</v>
       </c>
       <c r="K37" s="3"/>
     </row>
-    <row r="38" spans="1:11">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
         <v>52</v>
       </c>
@@ -1857,7 +1876,7 @@
       <c r="C38" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="D38" s="3">
+      <c r="D38" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E38" s="3" t="s">
@@ -1875,12 +1894,12 @@
       <c r="I38" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J38" s="4">
+      <c r="J38" s="4" t="n">
         <v>10755</v>
       </c>
       <c r="K38" s="3"/>
     </row>
-    <row r="39" spans="1:11">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
         <v>52</v>
       </c>
@@ -1890,7 +1909,7 @@
       <c r="C39" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="D39" s="3">
+      <c r="D39" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E39" s="3" t="s">
@@ -1908,14 +1927,14 @@
       <c r="I39" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J39" s="4">
+      <c r="J39" s="4" t="n">
         <v>10730</v>
       </c>
       <c r="K39" s="3" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="40" spans="1:11">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
         <v>52</v>
       </c>
@@ -1925,7 +1944,7 @@
       <c r="C40" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="D40" s="3">
+      <c r="D40" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E40" s="3" t="s">
@@ -1943,14 +1962,14 @@
       <c r="I40" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J40" s="4">
+      <c r="J40" s="4" t="n">
         <v>10730</v>
       </c>
       <c r="K40" s="3" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="41" spans="1:11">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
         <v>52</v>
       </c>
@@ -1960,7 +1979,7 @@
       <c r="C41" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="D41" s="3">
+      <c r="D41" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E41" s="3" t="s">
@@ -1978,12 +1997,12 @@
       <c r="I41" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J41" s="4">
+      <c r="J41" s="4" t="n">
         <v>10530</v>
       </c>
       <c r="K41" s="3"/>
     </row>
-    <row r="42" spans="1:11">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
         <v>52</v>
       </c>
@@ -1993,7 +2012,7 @@
       <c r="C42" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="D42" s="3">
+      <c r="D42" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E42" s="3" t="s">
@@ -2011,12 +2030,12 @@
       <c r="I42" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J42" s="4">
+      <c r="J42" s="4" t="n">
         <v>10770</v>
       </c>
       <c r="K42" s="3"/>
     </row>
-    <row r="43" spans="1:11">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
         <v>52</v>
       </c>
@@ -2026,7 +2045,7 @@
       <c r="C43" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="D43" s="3">
+      <c r="D43" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E43" s="3" t="s">
@@ -2044,12 +2063,12 @@
       <c r="I43" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J43" s="4">
+      <c r="J43" s="4" t="n">
         <v>10770</v>
       </c>
       <c r="K43" s="3"/>
     </row>
-    <row r="44" spans="1:11">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
         <v>52</v>
       </c>
@@ -2059,7 +2078,7 @@
       <c r="C44" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="D44" s="3">
+      <c r="D44" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E44" s="3" t="s">
@@ -2077,12 +2096,12 @@
       <c r="I44" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J44" s="4">
+      <c r="J44" s="4" t="n">
         <v>10730</v>
       </c>
       <c r="K44" s="3"/>
     </row>
-    <row r="45" spans="1:11">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
         <v>52</v>
       </c>
@@ -2092,7 +2111,7 @@
       <c r="C45" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="D45" s="3">
+      <c r="D45" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E45" s="3" t="s">
@@ -2110,12 +2129,12 @@
       <c r="I45" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J45" s="4">
+      <c r="J45" s="4" t="n">
         <v>10670</v>
       </c>
       <c r="K45" s="3"/>
     </row>
-    <row r="46" spans="1:11" ht="15" customHeight="1">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
         <v>52</v>
       </c>
@@ -2125,7 +2144,7 @@
       <c r="C46" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="D46" s="3">
+      <c r="D46" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E46" s="3" t="s">
@@ -2143,12 +2162,12 @@
       <c r="I46" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J46" s="4">
+      <c r="J46" s="4" t="n">
         <v>10730</v>
       </c>
       <c r="K46" s="6"/>
     </row>
-    <row r="47" spans="1:11">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
         <v>52</v>
       </c>
@@ -2158,7 +2177,7 @@
       <c r="C47" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="D47" s="3">
+      <c r="D47" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E47" s="3" t="s">
@@ -2176,12 +2195,12 @@
       <c r="I47" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J47" s="4">
+      <c r="J47" s="4" t="n">
         <v>10300</v>
       </c>
       <c r="K47" s="3"/>
     </row>
-    <row r="48" spans="1:11">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
         <v>52</v>
       </c>
@@ -2191,7 +2210,7 @@
       <c r="C48" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="D48" s="3">
+      <c r="D48" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E48" s="3" t="s">
@@ -2209,12 +2228,12 @@
       <c r="I48" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J48" s="4">
+      <c r="J48" s="4" t="n">
         <v>10720</v>
       </c>
       <c r="K48" s="3"/>
     </row>
-    <row r="49" spans="1:11">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
         <v>52</v>
       </c>
@@ -2224,7 +2243,7 @@
       <c r="C49" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="D49" s="3">
+      <c r="D49" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E49" s="3" t="s">
@@ -2242,12 +2261,12 @@
       <c r="I49" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J49" s="4">
+      <c r="J49" s="4" t="n">
         <v>10770</v>
       </c>
       <c r="K49" s="3"/>
     </row>
-    <row r="50" spans="1:11">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
         <v>52</v>
       </c>
@@ -2257,7 +2276,7 @@
       <c r="C50" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D50" s="3">
+      <c r="D50" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E50" s="3" t="s">
@@ -2275,12 +2294,12 @@
       <c r="I50" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J50" s="4">
+      <c r="J50" s="4" t="n">
         <v>10670</v>
       </c>
       <c r="K50" s="3"/>
     </row>
-    <row r="51" spans="1:11">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
         <v>52</v>
       </c>
@@ -2290,7 +2309,7 @@
       <c r="C51" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D51" s="3">
+      <c r="D51" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E51" s="3" t="s">
@@ -2308,12 +2327,12 @@
       <c r="I51" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J51" s="4">
+      <c r="J51" s="4" t="n">
         <v>10670</v>
       </c>
       <c r="K51" s="3"/>
     </row>
-    <row r="52" spans="1:11">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
         <v>52</v>
       </c>
@@ -2323,7 +2342,7 @@
       <c r="C52" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="D52" s="3">
+      <c r="D52" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E52" s="3" t="s">
@@ -2341,12 +2360,12 @@
       <c r="I52" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J52" s="4">
+      <c r="J52" s="4" t="n">
         <v>10300</v>
       </c>
       <c r="K52" s="3"/>
     </row>
-    <row r="53" spans="1:11">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
         <v>52</v>
       </c>
@@ -2356,7 +2375,7 @@
       <c r="C53" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="D53" s="3">
+      <c r="D53" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E53" s="3" t="s">
@@ -2374,14 +2393,14 @@
       <c r="I53" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J53" s="4">
+      <c r="J53" s="4" t="n">
         <v>3480</v>
       </c>
       <c r="K53" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="54" spans="1:11">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
         <v>52</v>
       </c>
@@ -2391,7 +2410,7 @@
       <c r="C54" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="D54" s="3">
+      <c r="D54" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E54" s="3" t="s">
@@ -2409,14 +2428,14 @@
       <c r="I54" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J54" s="4">
+      <c r="J54" s="4" t="n">
         <v>3480</v>
       </c>
       <c r="K54" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="55" spans="1:11">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
         <v>52</v>
       </c>
@@ -2426,7 +2445,7 @@
       <c r="C55" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="D55" s="3">
+      <c r="D55" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E55" s="3" t="s">
@@ -2449,7 +2468,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="56" spans="1:11">
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
         <v>52</v>
       </c>
@@ -2459,7 +2478,7 @@
       <c r="C56" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="D56" s="3">
+      <c r="D56" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E56" s="3" t="s">
@@ -2477,14 +2496,14 @@
       <c r="I56" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J56" s="4">
+      <c r="J56" s="4" t="n">
         <v>3460</v>
       </c>
       <c r="K56" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="57" spans="1:11">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
         <v>52</v>
       </c>
@@ -2494,7 +2513,7 @@
       <c r="C57" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="D57" s="3">
+      <c r="D57" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E57" s="3" t="s">
@@ -2512,14 +2531,14 @@
       <c r="I57" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J57" s="4">
+      <c r="J57" s="4" t="n">
         <v>3480</v>
       </c>
       <c r="K57" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="58" spans="1:11">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
         <v>52</v>
       </c>
@@ -2529,7 +2548,7 @@
       <c r="C58" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="D58" s="3">
+      <c r="D58" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E58" s="3" t="s">
@@ -2552,7 +2571,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="59" spans="1:11">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
         <v>52</v>
       </c>
@@ -2562,7 +2581,7 @@
       <c r="C59" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="D59" s="3">
+      <c r="D59" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E59" s="3" t="s">
@@ -2585,7 +2604,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="60" spans="1:11">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
         <v>52</v>
       </c>
@@ -2595,7 +2614,7 @@
       <c r="C60" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="D60" s="3">
+      <c r="D60" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E60" s="3" t="s">
@@ -2618,7 +2637,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="61" spans="1:11" ht="15" customHeight="1">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
         <v>52</v>
       </c>
@@ -2628,7 +2647,7 @@
       <c r="C61" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="D61" s="3">
+      <c r="D61" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E61" s="3" t="s">
@@ -2651,7 +2670,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="62" spans="1:11" ht="15" customHeight="1">
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
         <v>52</v>
       </c>
@@ -2661,7 +2680,7 @@
       <c r="C62" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="D62" s="3">
+      <c r="D62" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E62" s="3" t="s">
@@ -2684,7 +2703,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="63" spans="1:11" ht="15" customHeight="1">
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
         <v>52</v>
       </c>
@@ -2694,7 +2713,7 @@
       <c r="C63" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="D63" s="7">
+      <c r="D63" s="7" t="n">
         <v>1</v>
       </c>
       <c r="E63" s="7" t="s">
@@ -2712,12 +2731,12 @@
       <c r="I63" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="J63" s="8">
+      <c r="J63" s="8" t="n">
         <v>12980</v>
       </c>
       <c r="K63" s="9"/>
     </row>
-    <row r="64" spans="1:11">
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
         <v>52</v>
       </c>
@@ -2727,7 +2746,7 @@
       <c r="C64" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="D64" s="3">
+      <c r="D64" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E64" s="3" t="s">
@@ -2750,7 +2769,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="65" spans="1:11">
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="3" t="s">
         <v>52</v>
       </c>
@@ -2760,7 +2779,7 @@
       <c r="C65" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="D65" s="10">
+      <c r="D65" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E65" s="10" t="s">
@@ -2778,12 +2797,12 @@
       <c r="I65" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="J65" s="11">
+      <c r="J65" s="11" t="n">
         <v>10750</v>
       </c>
       <c r="K65" s="10"/>
     </row>
-    <row r="66" spans="1:11">
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
         <v>52</v>
       </c>
@@ -2793,7 +2812,7 @@
       <c r="C66" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="D66" s="3">
+      <c r="D66" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E66" s="3" t="s">
@@ -2816,7 +2835,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="67" spans="1:11">
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="3" t="s">
         <v>52</v>
       </c>
@@ -2826,7 +2845,7 @@
       <c r="C67" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="D67" s="3">
+      <c r="D67" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E67" s="3" t="s">
@@ -2849,7 +2868,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="68" spans="1:11">
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
         <v>52</v>
       </c>
@@ -2859,7 +2878,7 @@
       <c r="C68" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="D68" s="10">
+      <c r="D68" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E68" s="10" t="s">
@@ -2882,7 +2901,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="69" spans="1:11">
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="3" t="s">
         <v>52</v>
       </c>
@@ -2892,7 +2911,7 @@
       <c r="C69" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="D69" s="10">
+      <c r="D69" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E69" s="10" t="s">
@@ -2915,7 +2934,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="70" spans="1:11">
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
         <v>52</v>
       </c>
@@ -2925,7 +2944,7 @@
       <c r="C70" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="D70" s="10">
+      <c r="D70" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E70" s="10" t="s">
@@ -2941,12 +2960,12 @@
         <v>139</v>
       </c>
       <c r="I70" s="10"/>
-      <c r="J70" s="11">
+      <c r="J70" s="11" t="n">
         <v>16000</v>
       </c>
       <c r="K70" s="10"/>
     </row>
-    <row r="71" spans="1:11">
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="3" t="s">
         <v>52</v>
       </c>
@@ -2956,7 +2975,7 @@
       <c r="C71" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="D71" s="10">
+      <c r="D71" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E71" s="10" t="s">
@@ -2974,14 +2993,14 @@
       <c r="I71" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="J71" s="11">
+      <c r="J71" s="11" t="n">
         <v>10480</v>
       </c>
       <c r="K71" s="10" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="72" spans="1:11">
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="3"/>
       <c r="B72" s="10"/>
       <c r="C72" s="10"/>
@@ -2994,7 +3013,7 @@
       <c r="J72" s="10"/>
       <c r="K72" s="10"/>
     </row>
-    <row r="73" spans="1:11">
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
         <v>52</v>
       </c>
@@ -3004,7 +3023,7 @@
       <c r="C73" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D73" s="3">
+      <c r="D73" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E73" s="3" t="s">
@@ -3022,12 +3041,12 @@
       <c r="I73" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J73" s="4">
+      <c r="J73" s="4" t="n">
         <v>10755</v>
       </c>
       <c r="K73" s="3"/>
     </row>
-    <row r="74" spans="1:11">
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
         <v>52</v>
       </c>
@@ -3037,7 +3056,7 @@
       <c r="C74" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="D74" s="3">
+      <c r="D74" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E74" s="3" t="s">
@@ -3055,12 +3074,12 @@
       <c r="I74" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J74" s="4">
+      <c r="J74" s="4" t="n">
         <v>10755</v>
       </c>
       <c r="K74" s="3"/>
     </row>
-    <row r="75" spans="1:11">
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="3" t="s">
         <v>52</v>
       </c>
@@ -3070,7 +3089,7 @@
       <c r="C75" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D75" s="3">
+      <c r="D75" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E75" s="3" t="s">
@@ -3088,12 +3107,12 @@
       <c r="I75" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J75" s="4">
+      <c r="J75" s="4" t="n">
         <v>10755</v>
       </c>
       <c r="K75" s="3"/>
     </row>
-    <row r="76" spans="1:11">
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
         <v>52</v>
       </c>
@@ -3103,7 +3122,7 @@
       <c r="C76" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D76" s="3">
+      <c r="D76" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E76" s="3" t="s">
@@ -3121,12 +3140,12 @@
       <c r="I76" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J76" s="4">
+      <c r="J76" s="4" t="n">
         <v>10755</v>
       </c>
       <c r="K76" s="3"/>
     </row>
-    <row r="77" spans="1:11">
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="3" t="s">
         <v>52</v>
       </c>
@@ -3136,7 +3155,7 @@
       <c r="C77" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="D77" s="3">
+      <c r="D77" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E77" s="3" t="s">
@@ -3154,12 +3173,12 @@
       <c r="I77" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J77" s="4">
+      <c r="J77" s="4" t="n">
         <v>10770</v>
       </c>
       <c r="K77" s="3"/>
     </row>
-    <row r="78" spans="1:11">
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
         <v>52</v>
       </c>
@@ -3169,7 +3188,7 @@
       <c r="C78" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="D78" s="3">
+      <c r="D78" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E78" s="3" t="s">
@@ -3187,14 +3206,14 @@
       <c r="I78" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J78" s="4">
+      <c r="J78" s="4" t="n">
         <v>10720</v>
       </c>
       <c r="K78" s="3" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="79" spans="1:11">
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="3" t="s">
         <v>52</v>
       </c>
@@ -3204,7 +3223,7 @@
       <c r="C79" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="D79" s="3">
+      <c r="D79" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E79" s="3" t="s">
@@ -3222,12 +3241,12 @@
       <c r="I79" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="J79" s="4">
+      <c r="J79" s="4" t="n">
         <v>10750</v>
       </c>
       <c r="K79" s="3"/>
     </row>
-    <row r="80" spans="1:11">
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="3" t="s">
         <v>52</v>
       </c>
@@ -3237,7 +3256,7 @@
       <c r="C80" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="D80" s="3">
+      <c r="D80" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E80" s="3" t="s">
@@ -3255,12 +3274,12 @@
       <c r="I80" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J80" s="4">
+      <c r="J80" s="4" t="n">
         <v>10730</v>
       </c>
       <c r="K80" s="3"/>
     </row>
-    <row r="81" spans="1:11">
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="3" t="s">
         <v>52</v>
       </c>
@@ -3270,7 +3289,7 @@
       <c r="C81" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="D81" s="3">
+      <c r="D81" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E81" s="3" t="s">
@@ -3288,14 +3307,14 @@
       <c r="I81" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J81" s="4">
+      <c r="J81" s="4" t="n">
         <v>10500</v>
       </c>
       <c r="K81" s="3" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="82" spans="1:11">
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="3" t="s">
         <v>52</v>
       </c>
@@ -3305,7 +3324,7 @@
       <c r="C82" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="D82" s="3">
+      <c r="D82" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E82" s="3" t="s">
@@ -3323,14 +3342,14 @@
       <c r="I82" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J82" s="4">
+      <c r="J82" s="4" t="n">
         <v>10530</v>
       </c>
       <c r="K82" s="3" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="83" spans="1:11">
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="3"/>
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
@@ -3343,7 +3362,7 @@
       <c r="J83" s="4"/>
       <c r="K83" s="3"/>
     </row>
-    <row r="84" spans="1:11">
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
         <v>52</v>
       </c>
@@ -3353,7 +3372,7 @@
       <c r="C84" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="D84" s="3">
+      <c r="D84" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E84" s="3" t="s">
@@ -3371,12 +3390,12 @@
       <c r="I84" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J84" s="4">
+      <c r="J84" s="4" t="n">
         <v>10830</v>
       </c>
       <c r="K84" s="3"/>
     </row>
-    <row r="85" spans="1:11">
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="3" t="s">
         <v>52</v>
       </c>
@@ -3386,7 +3405,7 @@
       <c r="C85" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="D85" s="3">
+      <c r="D85" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E85" s="3" t="s">
@@ -3404,14 +3423,14 @@
       <c r="I85" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J85" s="4">
+      <c r="J85" s="4" t="n">
         <v>10730</v>
       </c>
       <c r="K85" s="3" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="86" spans="1:11">
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="3" t="s">
         <v>52</v>
       </c>
@@ -3421,7 +3440,7 @@
       <c r="C86" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="D86" s="3">
+      <c r="D86" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E86" s="3" t="s">
@@ -3444,7 +3463,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="87" spans="1:11">
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="3" t="s">
         <v>52</v>
       </c>
@@ -3454,7 +3473,7 @@
       <c r="C87" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="D87" s="3">
+      <c r="D87" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E87" s="3" t="s">
@@ -3477,7 +3496,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="88" spans="1:11">
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
         <v>52</v>
       </c>
@@ -3487,7 +3506,7 @@
       <c r="C88" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="D88" s="3">
+      <c r="D88" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E88" s="3" t="s">
@@ -3505,12 +3524,12 @@
       <c r="I88" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="J88" s="4">
+      <c r="J88" s="4" t="n">
         <v>16000</v>
       </c>
       <c r="K88" s="3"/>
     </row>
-    <row r="89" spans="1:11">
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="3" t="s">
         <v>52</v>
       </c>
@@ -3520,7 +3539,7 @@
       <c r="C89" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D89" s="3">
+      <c r="D89" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E89" s="3" t="s">
@@ -3538,12 +3557,12 @@
       <c r="I89" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J89" s="4">
+      <c r="J89" s="4" t="n">
         <v>10670</v>
       </c>
       <c r="K89" s="3"/>
     </row>
-    <row r="90" spans="1:11">
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="3" t="s">
         <v>52</v>
       </c>
@@ -3553,7 +3572,7 @@
       <c r="C90" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="D90" s="3">
+      <c r="D90" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E90" s="3" t="s">
@@ -3571,12 +3590,12 @@
       <c r="I90" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J90" s="4">
+      <c r="J90" s="4" t="n">
         <v>9720</v>
       </c>
       <c r="K90" s="3"/>
     </row>
-    <row r="91" spans="1:11">
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="3" t="s">
         <v>52</v>
       </c>
@@ -3586,7 +3605,7 @@
       <c r="C91" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="D91" s="3">
+      <c r="D91" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E91" s="3" t="s">
@@ -3604,14 +3623,14 @@
       <c r="I91" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J91" s="4">
+      <c r="J91" s="4" t="n">
         <v>10670</v>
       </c>
       <c r="K91" s="3" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="92" spans="1:11">
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
         <v>52</v>
       </c>
@@ -3621,7 +3640,7 @@
       <c r="C92" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="D92" s="3">
+      <c r="D92" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E92" s="3" t="s">
@@ -3639,12 +3658,12 @@
       <c r="I92" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J92" s="4">
+      <c r="J92" s="4" t="n">
         <v>10710</v>
       </c>
       <c r="K92" s="3"/>
     </row>
-    <row r="93" spans="1:11">
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="3" t="s">
         <v>52</v>
       </c>
@@ -3654,7 +3673,7 @@
       <c r="C93" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D93" s="3">
+      <c r="D93" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E93" s="3" t="s">
@@ -3672,12 +3691,12 @@
       <c r="I93" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J93" s="4">
+      <c r="J93" s="4" t="n">
         <v>10670</v>
       </c>
       <c r="K93" s="3"/>
     </row>
-    <row r="94" spans="1:11">
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
         <v>52</v>
       </c>
@@ -3687,7 +3706,7 @@
       <c r="C94" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="D94" s="3">
+      <c r="D94" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E94" s="3" t="s">
@@ -3705,12 +3724,12 @@
       <c r="I94" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J94" s="4">
+      <c r="J94" s="4" t="n">
         <v>10710</v>
       </c>
       <c r="K94" s="3"/>
     </row>
-    <row r="95" spans="1:11">
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="3" t="s">
         <v>52</v>
       </c>
@@ -3720,7 +3739,7 @@
       <c r="C95" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="D95" s="3">
+      <c r="D95" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E95" s="3" t="s">
@@ -3738,12 +3757,12 @@
       <c r="I95" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J95" s="4">
+      <c r="J95" s="4" t="n">
         <v>10715</v>
       </c>
       <c r="K95" s="3"/>
     </row>
-    <row r="96" spans="1:11">
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="3" t="s">
         <v>52</v>
       </c>
@@ -3753,7 +3772,7 @@
       <c r="C96" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="D96" s="3">
+      <c r="D96" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E96" s="3" t="s">
@@ -3776,7 +3795,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="97" spans="1:11">
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="3" t="s">
         <v>52</v>
       </c>
@@ -3786,7 +3805,7 @@
       <c r="C97" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="D97" s="3">
+      <c r="D97" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E97" s="3" t="s">
@@ -3809,7 +3828,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="98" spans="1:11">
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
         <v>52</v>
       </c>
@@ -3819,7 +3838,7 @@
       <c r="C98" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="D98" s="3">
+      <c r="D98" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E98" s="3" t="s">
@@ -3842,7 +3861,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="99" spans="1:11">
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="3" t="s">
         <v>52</v>
       </c>
@@ -3852,7 +3871,7 @@
       <c r="C99" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="D99" s="3">
+      <c r="D99" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E99" s="3" t="s">
@@ -3875,7 +3894,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="100" spans="1:11">
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="3" t="s">
         <v>52</v>
       </c>
@@ -3885,7 +3904,7 @@
       <c r="C100" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="D100" s="3">
+      <c r="D100" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E100" s="3" t="s">
@@ -3908,7 +3927,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="101" spans="1:11">
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="3" t="s">
         <v>52</v>
       </c>
@@ -3918,7 +3937,7 @@
       <c r="C101" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="D101" s="3">
+      <c r="D101" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E101" s="3" t="s">
@@ -3936,12 +3955,12 @@
       <c r="I101" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J101" s="4">
+      <c r="J101" s="4" t="n">
         <v>10830</v>
       </c>
       <c r="K101" s="3"/>
     </row>
-    <row r="102" spans="1:11">
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="3" t="s">
         <v>52</v>
       </c>
@@ -3951,7 +3970,7 @@
       <c r="C102" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="D102" s="3">
+      <c r="D102" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E102" s="3" t="s">
@@ -3969,12 +3988,12 @@
       <c r="I102" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J102" s="4">
+      <c r="J102" s="4" t="n">
         <v>3520</v>
       </c>
       <c r="K102" s="3"/>
     </row>
-    <row r="103" spans="1:11">
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="3" t="s">
         <v>52</v>
       </c>
@@ -3984,7 +4003,7 @@
       <c r="C103" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="D103" s="3">
+      <c r="D103" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E103" s="3"/>
@@ -3995,7 +4014,7 @@
       <c r="J103" s="4"/>
       <c r="K103" s="3"/>
     </row>
-    <row r="104" spans="1:11">
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="3" t="s">
         <v>52</v>
       </c>
@@ -4005,7 +4024,7 @@
       <c r="C104" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="D104" s="3">
+      <c r="D104" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E104" s="3" t="s">
@@ -4028,7 +4047,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="105" spans="1:11">
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="3" t="s">
         <v>52</v>
       </c>
@@ -4038,7 +4057,7 @@
       <c r="C105" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="D105" s="3">
+      <c r="D105" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E105" s="3" t="s">
@@ -4061,7 +4080,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="106" spans="1:11">
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="3" t="s">
         <v>52</v>
       </c>
@@ -4071,7 +4090,7 @@
       <c r="C106" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="D106" s="3">
+      <c r="D106" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E106" s="3" t="s">
@@ -4092,7 +4111,7 @@
       <c r="J106" s="4"/>
       <c r="K106" s="3"/>
     </row>
-    <row r="107" spans="1:11">
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="3"/>
       <c r="B107" s="3"/>
       <c r="C107" s="3"/>
@@ -4105,7 +4124,7 @@
       <c r="J107" s="4"/>
       <c r="K107" s="3"/>
     </row>
-    <row r="108" spans="1:11">
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="3" t="s">
         <v>52</v>
       </c>
@@ -4115,7 +4134,7 @@
       <c r="C108" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="D108" s="3">
+      <c r="D108" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E108" s="3" t="s">
@@ -4136,7 +4155,7 @@
       <c r="J108" s="4"/>
       <c r="K108" s="3"/>
     </row>
-    <row r="109" spans="1:11">
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="3" t="s">
         <v>52</v>
       </c>
@@ -4146,7 +4165,7 @@
       <c r="C109" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="D109" s="3">
+      <c r="D109" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E109" s="3" t="s">
@@ -4167,7 +4186,7 @@
       <c r="J109" s="3"/>
       <c r="K109" s="3"/>
     </row>
-    <row r="110" spans="1:11">
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="3" t="s">
         <v>52</v>
       </c>
@@ -4177,7 +4196,7 @@
       <c r="C110" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="D110" s="3">
+      <c r="D110" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E110" s="3" t="s">
@@ -4198,7 +4217,7 @@
       <c r="J110" s="4"/>
       <c r="K110" s="3"/>
     </row>
-    <row r="111" spans="1:11">
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="3" t="s">
         <v>52</v>
       </c>
@@ -4208,7 +4227,7 @@
       <c r="C111" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="D111" s="3">
+      <c r="D111" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E111" s="3" t="s">
@@ -4226,12 +4245,12 @@
       <c r="I111" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J111" s="4">
+      <c r="J111" s="4" t="n">
         <v>10550</v>
       </c>
       <c r="K111" s="3"/>
     </row>
-    <row r="112" spans="1:11">
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="3" t="s">
         <v>52</v>
       </c>
@@ -4241,7 +4260,7 @@
       <c r="C112" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="D112" s="3">
+      <c r="D112" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E112" s="3" t="s">
@@ -4262,7 +4281,7 @@
       <c r="J112" s="3"/>
       <c r="K112" s="3"/>
     </row>
-    <row r="113" spans="1:11">
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="3" t="s">
         <v>52</v>
       </c>
@@ -4272,7 +4291,7 @@
       <c r="C113" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="D113" s="3">
+      <c r="D113" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E113" s="3" t="s">
@@ -4293,7 +4312,7 @@
       <c r="J113" s="3"/>
       <c r="K113" s="3"/>
     </row>
-    <row r="114" spans="1:11">
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="3" t="s">
         <v>52</v>
       </c>
@@ -4303,7 +4322,7 @@
       <c r="C114" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="D114" s="3">
+      <c r="D114" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E114" s="3" t="s">
@@ -4324,7 +4343,7 @@
       <c r="J114" s="3"/>
       <c r="K114" s="3"/>
     </row>
-    <row r="115" spans="1:11">
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="3"/>
       <c r="B115" s="3"/>
       <c r="C115" s="3"/>
@@ -4337,7 +4356,7 @@
       <c r="J115" s="3"/>
       <c r="K115" s="3"/>
     </row>
-    <row r="116" spans="1:11">
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="3" t="s">
         <v>52</v>
       </c>
@@ -4347,7 +4366,7 @@
       <c r="C116" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="D116" s="3">
+      <c r="D116" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E116" s="3" t="s">
@@ -4365,12 +4384,12 @@
       <c r="I116" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="J116" s="4">
+      <c r="J116" s="4" t="n">
         <v>14000</v>
       </c>
       <c r="K116" s="3"/>
     </row>
-    <row r="117" spans="1:11">
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="3" t="s">
         <v>52</v>
       </c>
@@ -4380,7 +4399,7 @@
       <c r="C117" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="D117" s="3">
+      <c r="D117" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E117" s="3" t="s">
@@ -4398,14 +4417,14 @@
       <c r="I117" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="J117" s="4">
+      <c r="J117" s="4" t="n">
         <v>10550</v>
       </c>
       <c r="K117" s="3" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="118" spans="1:11">
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="3" t="s">
         <v>52</v>
       </c>
@@ -4415,7 +4434,7 @@
       <c r="C118" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="D118" s="3">
+      <c r="D118" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E118" s="3" t="s">
@@ -4436,7 +4455,7 @@
       <c r="J118" s="3"/>
       <c r="K118" s="3"/>
     </row>
-    <row r="119" spans="1:11">
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="3" t="s">
         <v>52</v>
       </c>
@@ -4446,7 +4465,7 @@
       <c r="C119" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="D119" s="3">
+      <c r="D119" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E119" s="3" t="s">
@@ -4464,12 +4483,12 @@
       <c r="I119" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J119" s="4">
+      <c r="J119" s="4" t="n">
         <v>10550</v>
       </c>
       <c r="K119" s="3"/>
     </row>
-    <row r="120" spans="1:11">
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="3" t="s">
         <v>52</v>
       </c>
@@ -4479,7 +4498,7 @@
       <c r="C120" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="D120" s="3">
+      <c r="D120" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E120" s="3" t="s">
@@ -4497,12 +4516,12 @@
       <c r="I120" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J120" s="4">
+      <c r="J120" s="4" t="n">
         <v>10550</v>
       </c>
       <c r="K120" s="3"/>
     </row>
-    <row r="121" spans="1:11">
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="3" t="s">
         <v>52</v>
       </c>
@@ -4512,7 +4531,7 @@
       <c r="C121" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="D121" s="3">
+      <c r="D121" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E121" s="3" t="s">
@@ -4530,13 +4549,18 @@
       <c r="I121" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J121" s="4">
+      <c r="J121" s="4" t="n">
         <v>10580</v>
       </c>
       <c r="K121" s="3"/>
     </row>
   </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>